<commit_message>
Sync 38 sent + send Mowbray/Rondebosch 2026-10-07-1722
</commit_message>
<xml_diff>
--- a/inbox/areas_contacts.xlsx
+++ b/inbox/areas_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="55">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -560,6 +560,9 @@
       <c r="D3" t="s">
         <v>50</v>
       </c>
+      <c r="E3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
@@ -574,6 +577,9 @@
       <c r="D4" t="s">
         <v>50</v>
       </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
@@ -588,6 +594,9 @@
       <c r="D5" t="s">
         <v>50</v>
       </c>
+      <c r="E5" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
@@ -602,6 +611,9 @@
       <c r="D6" t="s">
         <v>50</v>
       </c>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
@@ -616,6 +628,9 @@
       <c r="D7" t="s">
         <v>50</v>
       </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
@@ -630,6 +645,9 @@
       <c r="D8" t="s">
         <v>50</v>
       </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
@@ -643,6 +661,9 @@
       </c>
       <c r="D9" t="s">
         <v>50</v>
+      </c>
+      <c r="E9" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:5">

</xml_diff>

<commit_message>
Send Mowbray batch 2026-10-07-1723
</commit_message>
<xml_diff>
--- a/inbox/areas_contacts.xlsx
+++ b/inbox/areas_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="55">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -679,6 +679,9 @@
       <c r="D10" t="s">
         <v>50</v>
       </c>
+      <c r="E10" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">

</xml_diff>

<commit_message>
Send pending contacts 2026-10-07-1731
</commit_message>
<xml_diff>
--- a/inbox/areas_contacts.xlsx
+++ b/inbox/areas_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="55">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -696,6 +696,9 @@
       <c r="D11" t="s">
         <v>50</v>
       </c>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
@@ -710,6 +713,9 @@
       <c r="D12" t="s">
         <v>50</v>
       </c>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
@@ -724,6 +730,9 @@
       <c r="D13" t="s">
         <v>50</v>
       </c>
+      <c r="E13" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
@@ -738,6 +747,9 @@
       <c r="D14" t="s">
         <v>50</v>
       </c>
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
@@ -752,6 +764,9 @@
       <c r="D15" t="s">
         <v>50</v>
       </c>
+      <c r="E15" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
@@ -766,8 +781,11 @@
       <c r="D16" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -780,8 +798,11 @@
       <c r="D17" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -794,8 +815,11 @@
       <c r="D18" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -809,7 +833,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Send Mowbray and Rondebosch batch 2026-10-07-1733
</commit_message>
<xml_diff>
--- a/inbox/areas_contacts.xlsx
+++ b/inbox/areas_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="55">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -832,6 +832,9 @@
       <c r="D19" t="s">
         <v>52</v>
       </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
@@ -845,6 +848,9 @@
       </c>
       <c r="D20" t="s">
         <v>52</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>